<commit_message>
Re-baseline dump artifacts against released v0.7.2 XLL
</commit_message>
<xml_diff>
--- a/excel/actuarial_add_in.xlsx
+++ b/excel/actuarial_add_in.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matth\actuarial_dump_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9DECFAE-8E63-4177-93E7-46E6397C26FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB62A974-589C-4C64-B6B3-E2F7851D7F87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -14169,7 +14169,7 @@
       </c>
       <c r="B3" t="str">
         <f>_xll.ACT_VERSION()</f>
-        <v>0.7.1</v>
+        <v>0.7.2</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -14201,7 +14201,7 @@
       </c>
       <c r="B8" t="str">
         <f>_xll.ACT_VERSION()</f>
-        <v>0.7.1</v>
+        <v>0.7.2</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -14228,7 +14228,7 @@
       </c>
       <c r="B11">
         <f>_xll.ACT_COMMIT_COUNT()</f>
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -14237,7 +14237,7 @@
       </c>
       <c r="B12" t="str">
         <f>_xll.ACT_COMMIT_INFO(1, "message")</f>
-        <v>Patch: replace `int? seed = null` with `object seed = null` + ResolveSeed helper across 13 stochastic functions. ExcelDna 1.9.0 mis-marshals `int?` parameters from Excel even though direct C# calls work — every cell calling the affected functions returned #VALUE! pre-fix (373 cells in the dump test).</v>
+        <v>Workbook polish + Experimental retagging. Mack-SE reference column corrected; Cat Modeling EP-curve table populated; Latest Cumulative restored as a formula; Copulas sheet gains Gaussian/Clayton/Frank/Gumbel sections; Interpolation chart shows interpolated overlay; all charts switched from smooth to straight lines; array formulas promoted via Formula2 to spill correctly. `Actuarial.Aggregate`/`Reinsurance` cat-modelling and return-period functions retagged Experimental to match Copulas/Bootstrap.</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -18723,7 +18723,7 @@
       </c>
       <c r="B304" t="str">
         <f>_xll.ACT_VERSION()</f>
-        <v>0.7.1</v>
+        <v>0.7.2</v>
       </c>
       <c r="C304" t="s">
         <v>373</v>
@@ -18759,7 +18759,7 @@
       </c>
       <c r="B307">
         <f>_xll.ACT_COMMIT_COUNT()</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C307" t="s">
         <v>379</v>
@@ -18771,7 +18771,7 @@
       </c>
       <c r="B308" t="str">
         <f>_xll.ACT_COMMIT_INFO(1, "hash")</f>
-        <v>v0.7.1</v>
+        <v>v0.7.2</v>
       </c>
       <c r="C308" t="s">
         <v>381</v>
@@ -18795,7 +18795,7 @@
       </c>
       <c r="B310" t="str">
         <f>_xll.ACT_COMMIT_INFO(1, "message")</f>
-        <v>Patch: replace `int? seed = null` with `object seed = null` + ResolveSeed helper across 13 stochastic functions. ExcelDna 1.9.0 mis-marshals `int?` parameters from Excel even though direct C# calls work — every cell calling the affected functions returned #VALUE! pre-fix (373 cells in the dump test).</v>
+        <v>Workbook polish + Experimental retagging. Mack-SE reference column corrected; Cat Modeling EP-curve table populated; Latest Cumulative restored as a formula; Copulas sheet gains Gaussian/Clayton/Frank/Gumbel sections; Interpolation chart shows interpolated overlay; all charts switched from smooth to straight lines; array formulas promoted via Formula2 to spill correctly. `Actuarial.Aggregate`/`Reinsurance` cat-modelling and return-period functions retagged Experimental to match Copulas/Bootstrap.</v>
       </c>
       <c r="C310" t="s">
         <v>383</v>

</xml_diff>

<commit_message>
v0.8.0: multi-target net48 + net8.0-windows
</commit_message>
<xml_diff>
--- a/excel/actuarial_add_in.xlsx
+++ b/excel/actuarial_add_in.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matth\actuarial_dump_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E942EA-C49D-4CD8-B95C-F5B0E861EBD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A4F6CD6-8394-4F1D-BF47-6E4236B4AD1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2188,7 +2188,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-45B8-4BF9-9E81-C415D07AE718}"/>
+              <c16:uniqueId val="{00000000-E0BD-4811-9134-639F430D872D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2402,7 +2402,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-7DCD-4479-B62D-9CF771CC3191}"/>
+              <c16:uniqueId val="{00000000-B230-410A-89AA-494432E71D83}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2617,7 +2617,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-AC1D-46F4-83C8-8B81DAE90636}"/>
+              <c16:uniqueId val="{00000000-9C02-41DF-82E7-A07DFEB710B3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2832,7 +2832,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-264A-467B-A587-E37FB57A76C5}"/>
+              <c16:uniqueId val="{00000000-AAB4-4FB9-A9E6-CFE88F281A2B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3047,7 +3047,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-8ED5-4E12-93CD-6E9D7ACDCEB9}"/>
+              <c16:uniqueId val="{00000000-AA43-4357-81B3-326B7C9FA519}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3262,7 +3262,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-865F-4874-A56D-AC545B990398}"/>
+              <c16:uniqueId val="{00000000-1C22-48D4-8B57-7DC3C462AE9C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3483,7 +3483,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-B721-4EB4-B4F5-093155CFB33A}"/>
+              <c16:uniqueId val="{00000000-941E-43CF-B05C-286C25D9A673}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3705,7 +3705,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-1BF0-4C94-BEB7-6099BE6ACBD9}"/>
+              <c16:uniqueId val="{00000000-0225-4945-89F6-74375D25044F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3927,7 +3927,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-AC99-4A35-9E5C-E84ED9F55408}"/>
+              <c16:uniqueId val="{00000000-F899-49AC-932A-4AC08FCC4887}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4149,7 +4149,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-CC66-4D67-91F4-F05E362498F9}"/>
+              <c16:uniqueId val="{00000000-E610-430D-9236-9692E8F6B073}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4377,7 +4377,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-7F31-4572-8E9B-3056984E7AAB}"/>
+              <c16:uniqueId val="{00000000-74E9-4CB8-A574-9AE43129D506}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4605,7 +4605,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-164F-45AD-8F96-2A8D16A4A979}"/>
+              <c16:uniqueId val="{00000000-F411-49AC-A0F5-C53EF11E2A95}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4826,7 +4826,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-26E5-41F1-9FBC-0CE042F7B13F}"/>
+              <c16:uniqueId val="{00000000-1903-433D-B8A0-2888B7B982AF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5042,7 +5042,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C7B4-4A06-B8F5-338ED2CE797D}"/>
+              <c16:uniqueId val="{00000000-B129-47F4-A45C-90816530EE5C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5252,7 +5252,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-1ED6-47F6-8D7C-002E86B57067}"/>
+              <c16:uniqueId val="{00000000-5DE2-40CE-911B-5F83C65F228A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5474,7 +5474,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-B79C-40B6-80B4-E5648F62D56F}"/>
+              <c16:uniqueId val="{00000000-438B-45B4-AA9A-E3EF27B5E84C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5695,7 +5695,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-8E80-45F3-8054-8175D5219AAE}"/>
+              <c16:uniqueId val="{00000000-8FBC-4D6B-AAF4-D12552841B10}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5916,7 +5916,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-13F8-4808-8B6C-300499F15886}"/>
+              <c16:uniqueId val="{00000000-9B5E-44DD-B819-01D86529AA39}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6146,7 +6146,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-E00B-4201-B22E-862A04058E8B}"/>
+              <c16:uniqueId val="{00000000-8113-470E-BE9F-F977C71D6FDA}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6254,7 +6254,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-E00B-4201-B22E-862A04058E8B}"/>
+              <c16:uniqueId val="{00000001-8113-470E-BE9F-F977C71D6FDA}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6362,7 +6362,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-E00B-4201-B22E-862A04058E8B}"/>
+              <c16:uniqueId val="{00000002-8113-470E-BE9F-F977C71D6FDA}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6470,7 +6470,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-E00B-4201-B22E-862A04058E8B}"/>
+              <c16:uniqueId val="{00000003-8113-470E-BE9F-F977C71D6FDA}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6578,7 +6578,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-E00B-4201-B22E-862A04058E8B}"/>
+              <c16:uniqueId val="{00000004-8113-470E-BE9F-F977C71D6FDA}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6787,7 +6787,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-2E9E-4768-856C-AE21EFB80DCD}"/>
+              <c16:uniqueId val="{00000000-0094-44C2-90C3-BB5AF971277F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6878,7 +6878,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-2E9E-4768-856C-AE21EFB80DCD}"/>
+              <c16:uniqueId val="{00000001-0094-44C2-90C3-BB5AF971277F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7109,7 +7109,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-93C6-4B57-BD0B-A9C012E4057A}"/>
+              <c16:uniqueId val="{00000000-E712-4FF2-9A65-D6EC419C80EA}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7338,7 +7338,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-8A88-469C-AD60-552EA2C9B11D}"/>
+              <c16:uniqueId val="{00000000-F5A0-4F24-9BCB-EEDB6DA9258A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7442,7 +7442,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-8A88-469C-AD60-552EA2C9B11D}"/>
+              <c16:uniqueId val="{00000001-F5A0-4F24-9BCB-EEDB6DA9258A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7681,7 +7681,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-F40C-458E-8C6D-43A52CB3A190}"/>
+              <c16:uniqueId val="{00000000-0DDB-4D52-A4CB-E5840C1CB65B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7908,7 +7908,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-896B-4A49-B9A4-537402FFF37A}"/>
+              <c16:uniqueId val="{00000000-6078-4F5C-A0B9-2F09C957609D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -8678,7 +8678,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-F27E-43F3-AA22-A9DB0B287E0E}"/>
+              <c16:uniqueId val="{00000000-44F0-4E68-9150-D4D7622CFA5C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -9148,7 +9148,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-3D89-467D-BBAB-CA578F281071}"/>
+              <c16:uniqueId val="{00000000-FE40-4837-B73E-ACFD5C27B0DE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -9618,7 +9618,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-A7D3-46CA-9E99-04C6A29C3433}"/>
+              <c16:uniqueId val="{00000000-3D2C-450B-8879-24E81AFD7915}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -10088,7 +10088,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-0DD0-45CE-8398-039FADB9FD4B}"/>
+              <c16:uniqueId val="{00000000-B342-44A3-B1CB-A88D18B535D8}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -10253,7 +10253,7 @@
                   <c:v>0.42463282830797527</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.35380375198453234</c:v>
+                  <c:v>0.35380375198453229</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0.44659383954294735</c:v>
@@ -10355,7 +10355,7 @@
                   <c:v>0.51050373743944277</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>0.14401509733294562</c:v>
+                  <c:v>0.14401509733294554</c:v>
                 </c:pt>
                 <c:pt idx="38">
                   <c:v>0.96172356733895836</c:v>
@@ -10412,7 +10412,7 @@
                   <c:v>0.43659012860129937</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.2931304282767539</c:v>
+                  <c:v>0.29313042827675378</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0.26771098674491789</c:v>
@@ -10469,7 +10469,7 @@
                   <c:v>0.13870552160293764</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.60361747146042066</c:v>
+                  <c:v>0.60361747146042077</c:v>
                 </c:pt>
                 <c:pt idx="23">
                   <c:v>0.80369712894477241</c:v>
@@ -10514,7 +10514,7 @@
                   <c:v>0.50509787790445482</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>6.1403171916247834E-2</c:v>
+                  <c:v>6.1403171916247806E-2</c:v>
                 </c:pt>
                 <c:pt idx="38">
                   <c:v>0.84179786840587534</c:v>
@@ -10558,7 +10558,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-0F6A-45A6-9218-413D9D1A0A93}"/>
+              <c16:uniqueId val="{00000000-786F-4540-B98F-D513A8A6421E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -10907,7 +10907,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-1DB3-40CC-A3C9-B31F55912BD0}"/>
+              <c16:uniqueId val="{00000000-4891-43A4-8F5C-CB66CA8175C8}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -11100,7 +11100,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-63AA-4F63-BC80-A127376EC4E7}"/>
+              <c16:uniqueId val="{00000000-BF3C-45D0-9379-17477E3E7D6A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -11321,7 +11321,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-E939-4DB8-89B7-5754C90DF35A}"/>
+              <c16:uniqueId val="{00000000-15CD-42EC-88D3-A6E8E3FAACD4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -11536,7 +11536,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-A1F3-4E45-84A6-30D9383984B2}"/>
+              <c16:uniqueId val="{00000000-4854-4029-B95D-02C4713E05F0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -11751,7 +11751,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-30E3-4A55-B3DB-ACF3B0F29405}"/>
+              <c16:uniqueId val="{00000000-97AB-456C-BF6A-932C6E90449D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -11966,7 +11966,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-3F5E-4743-97C5-D6B5309B5293}"/>
+              <c16:uniqueId val="{00000000-14C3-41E2-AF14-1510D9576B98}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -12193,7 +12193,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-A648-4874-A451-93B7F1517430}"/>
+              <c16:uniqueId val="{00000000-B822-4402-B741-E0B74652C8CF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -12403,7 +12403,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-7BD9-41A3-9616-7907BC2832C7}"/>
+              <c16:uniqueId val="{00000000-A7CC-4C90-B441-405CAE9AFCD1}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -13966,7 +13966,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -13986,7 +13986,7 @@
       </c>
       <c r="B3" t="str">
         <f>_xll.ACT_VERSION()</f>
-        <v>0.7.3</v>
+        <v>0.8.0</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -13995,7 +13995,7 @@
       </c>
       <c r="B4" t="str">
         <f>_xll.ACT_BUILD_DATE()</f>
-        <v>2026-05-04</v>
+        <v>2026-05-05</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -14018,7 +14018,7 @@
       </c>
       <c r="B8" t="str">
         <f>_xll.ACT_VERSION()</f>
-        <v>0.7.3</v>
+        <v>0.8.0</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -14027,7 +14027,7 @@
       </c>
       <c r="B9" t="str">
         <f>_xll.ACT_BUILD_DATE()</f>
-        <v>2026-05-04</v>
+        <v>2026-05-05</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -14045,7 +14045,7 @@
       </c>
       <c r="B11">
         <f>_xll.ACT_COMMIT_COUNT()</f>
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -14054,7 +14054,7 @@
       </c>
       <c r="B12" t="str">
         <f>_xll.ACT_COMMIT_INFO(1, "message")</f>
-        <v>Bundles five post-v0.7.2 fixes for the public surface: Cat Modeling SPILL collision (OEP/AEP curves now sit side-by-side with full 1000-row clearance, confused static Example 2 dropped); dump-iteration ordering (post-Formula2 errors now surface in dump JSON instead of silently shipping); Versions tab spills `=ACT_COMMIT_HISTORY()` live from the XLL instead of a stale `git log` snapshot; CHANGELOG.md / CONTRIBUTING.md / docs/DEVELOPING.md pulled out of the public repo (release notes live in this method + GitHub Releases).</v>
+        <v>Multi-target net48 + net8.0-windows. Default release asset (`AddIn64-packed.xll`) now targets .NET Framework 4.8 — preinstalled on every Windows 10 1903+ / Windows 11, so installing the add-in no longer requires a runtime download. A .NET 8 perf variant ships alongside as `AddIn64-packed-net8.xll` for users who install the .NET 8 Desktop Runtime; same C# code, modern JIT and SIMD codegen on heavy stochastic workloads. Root cause of the long-standing v0.5.x .NET 8 hosting failure identified: ExcelDna 1.9.0's host shim formats its own runtimeconfig.json from the `.dna` file's RuntimeVersion attribute, which was set to `v4.0` (causing the host to launch .NET 6 and reject the net8 user assembly). MSBuild XmlPoke target now rewrites it to `v8.0` for the net8 build only.</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -14064,7 +14064,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="str" cm="1">
-        <f t="array" ref="A15:C30">_xll.ACT_COMMIT_HISTORY()</f>
+        <f t="array" ref="A15:C31">_xll.ACT_COMMIT_HISTORY()</f>
         <v>Commit</v>
       </c>
       <c r="B15" t="str">
@@ -14076,166 +14076,177 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
-        <v>v0.7.3</v>
+        <v>v0.8.0</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-05-04</v>
+        <v>2026-05-05</v>
       </c>
       <c r="C16" t="str">
-        <v>Bundles five post-v0.7.2 fixes for the public surface: Cat Modeling SPILL collision (OEP/AEP curves now sit side-by-side with full 1000-row clearance, confused static Example 2 dropped); dump-iteration ordering (post-Formula2 errors now surface in dump JSON instead of silently shipping); Versions tab spills `=ACT_COMMIT_HISTORY()` live from the XLL instead of a stale `git log` snapshot; CHANGELOG.md / CONTRIBUTING.md / docs/DEVELOPING.md pulled out of the public repo (release notes live in this method + GitHub Releases).</v>
+        <v>Multi-target net48 + net8.0-windows. Default release asset (`AddIn64-packed.xll`) now targets .NET Framework 4.8 — preinstalled on every Windows 10 1903+ / Windows 11, so installing the add-in no longer requires a runtime download. A .NET 8 perf variant ships alongside as `AddIn64-packed-net8.xll` for users who install the .NET 8 Desktop Runtime; same C# code, modern JIT and SIMD codegen on heavy stochastic workloads. Root cause of the long-standing v0.5.x .NET 8 hosting failure identified: ExcelDna 1.9.0's host shim formats its own runtimeconfig.json from the `.dna` file's RuntimeVersion attribute, which was set to `v4.0` (causing the host to launch .NET 6 and reject the net8 user assembly). MSBuild XmlPoke target now rewrites it to `v8.0` for the net8 build only.</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="str">
-        <v>v0.7.2</v>
+        <v>v0.7.3</v>
       </c>
       <c r="B17" t="str">
         <v>2026-05-04</v>
       </c>
       <c r="C17" t="str">
-        <v>Workbook polish + Experimental retagging. Mack-SE reference column corrected; Cat Modeling EP-curve table populated; Latest Cumulative restored as a formula; Copulas sheet gains Gaussian/Clayton/Frank/Gumbel sections; Interpolation chart shows interpolated overlay; all charts switched from smooth to straight lines; array formulas promoted via Formula2 to spill correctly. `Actuarial.Aggregate`/`Reinsurance` cat-modelling and return-period functions retagged Experimental to match Copulas/Bootstrap.</v>
+        <v>Bundles five post-v0.7.2 fixes for the public surface: Cat Modeling SPILL collision (OEP/AEP curves now sit side-by-side with full 1000-row clearance, confused static Example 2 dropped); dump-iteration ordering (post-Formula2 errors now surface in dump JSON instead of silently shipping); Versions tab spills `=ACT_COMMIT_HISTORY()` live from the XLL instead of a stale `git log` snapshot; CHANGELOG.md / CONTRIBUTING.md / docs/DEVELOPING.md pulled out of the public repo (release notes live in this method + GitHub Releases).</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
-        <v>v0.7.1</v>
+        <v>v0.7.2</v>
       </c>
       <c r="B18" t="str">
         <v>2026-05-04</v>
       </c>
       <c r="C18" t="str">
-        <v>Patch: replace `int? seed = null` with `object seed = null` + ResolveSeed helper across 13 stochastic functions. ExcelDna 1.9.0 mis-marshals `int?` parameters from Excel even though direct C# calls work — every cell calling the affected functions returned #VALUE! pre-fix (373 cells in the dump test).</v>
+        <v>Workbook polish + Experimental retagging. Mack-SE reference column corrected; Cat Modeling EP-curve table populated; Latest Cumulative restored as a formula; Copulas sheet gains Gaussian/Clayton/Frank/Gumbel sections; Interpolation chart shows interpolated overlay; all charts switched from smooth to straight lines; array formulas promoted via Formula2 to spill correctly. `Actuarial.Aggregate`/`Reinsurance` cat-modelling and return-period functions retagged Experimental to match Copulas/Bootstrap.</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="str">
-        <v>v0.7.0</v>
+        <v>v0.7.1</v>
       </c>
       <c r="B19" t="str">
         <v>2026-05-04</v>
       </c>
       <c r="C19" t="str">
-        <v>Breaking: dropped Cape Cod, triangle-utility, calendar-adjust, weighted-average functions (9 in total). Added Mack factor SE / BF / CL_LATEST formulas to spreadsheet; harness now exercises every C# function (174); notebook reconciles every non-trivial function against scipy/Klugman/Bernegger references.</v>
+        <v>Patch: replace `int? seed = null` with `object seed = null` + ResolveSeed helper across 13 stochastic functions. ExcelDna 1.9.0 mis-marshals `int?` parameters from Excel even though direct C# calls work — every cell calling the affected functions returned #VALUE! pre-fix (373 cells in the dump test).</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="str">
-        <v>v0.6.0</v>
+        <v>v0.7.0</v>
       </c>
       <c r="B20" t="str">
         <v>2026-05-04</v>
       </c>
       <c r="C20" t="str">
-        <v>Internal cleanups: split Distributions.cs (1686 lines) and ChainLadder.cs (1510 lines) into focused partial-class files; standardised inline string-error returns to ExcelError.ExcelErrorValue (24 sites); test harness now exits non-zero on assertion failures.</v>
+        <v>Breaking: dropped Cape Cod, triangle-utility, calendar-adjust, weighted-average functions (9 in total). Added Mack factor SE / BF / CL_LATEST formulas to spreadsheet; harness now exercises every C# function (174); notebook reconciles every non-trivial function against scipy/Klugman/Bernegger references.</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
-        <v>v0.5.4</v>
+        <v>v0.6.0</v>
       </c>
       <c r="B21" t="str">
         <v>2026-05-04</v>
       </c>
       <c r="C21" t="str">
-        <v>Patch: ACT_EXPOSURE_MBBEFD numerical stability — rewrote without explicit `a` to fix NaN at SwissRe c=5 (b&lt;1, b^g underflow) and a 4th-decimal precision loss at c=3.</v>
+        <v>Internal cleanups: split Distributions.cs (1686 lines) and ChainLadder.cs (1510 lines) into focused partial-class files; standardised inline string-error returns to ExcelError.ExcelErrorValue (24 sites); test harness now exits non-zero on assertion failures.</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
-        <v>v0.5.3</v>
+        <v>v0.5.4</v>
       </c>
       <c r="B22" t="str">
         <v>2026-05-04</v>
       </c>
       <c r="C22" t="str">
-        <v>Patch: revert to net6.0-windows — neither ExcelDna 1.9.0 nor 1.10-preview4 reliably hosted .NET 8 in Excel. Keeps int? from 1.9; net6 path is known-good.</v>
+        <v>Patch: ACT_EXPOSURE_MBBEFD numerical stability — rewrote without explicit `a` to fix NaN at SwissRe c=5 (b&lt;1, b^g underflow) and a 4th-decimal precision loss at c=3.</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
-        <v>v0.5.2</v>
+        <v>v0.5.3</v>
       </c>
       <c r="B23" t="str">
         <v>2026-05-04</v>
       </c>
       <c r="C23" t="str">
-        <v>Patch: tried ExcelDna.AddIn 1.10-preview4 to fix .NET 8 hosting (didn't work).</v>
+        <v>Patch: revert to net6.0-windows — neither ExcelDna 1.9.0 nor 1.10-preview4 reliably hosted .NET 8 in Excel. Keeps int? from 1.9; net6 path is known-good.</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
-        <v>v0.5.1</v>
+        <v>v0.5.2</v>
       </c>
       <c r="B24" t="str">
-        <v>2026-05-03</v>
+        <v>2026-05-04</v>
       </c>
       <c r="C24" t="str">
-        <v>Patch: drop legacy RuntimeVersion="v4.0" from .dna manifest (necessary but not sufficient — see v0.5.2).</v>
+        <v>Patch: tried ExcelDna.AddIn 1.10-preview4 to fix .NET 8 hosting (didn't work).</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="str">
-        <v>v0.5.0</v>
+        <v>v0.5.1</v>
       </c>
       <c r="B25" t="str">
         <v>2026-05-03</v>
       </c>
       <c r="C25" t="str">
-        <v>Numerical fixes (LAYER_RATE, ILF_PARETO with xm, SWISSRE→Bernegger, AGGREGATE_TVAR); ExcelDna 1.9 + net8.0-windows; nullable seed; copula error handling.</v>
+        <v>Patch: drop legacy RuntimeVersion="v4.0" from .dna manifest (necessary but not sufficient — see v0.5.2).</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="str">
-        <v>v0.4.0</v>
+        <v>v0.5.0</v>
       </c>
       <c r="B26" t="str">
-        <v>2026-05-02</v>
+        <v>2026-05-03</v>
       </c>
       <c r="C26" t="str">
-        <v>GLM hat matrix bootstrap; Aggregate Claims formula fix; broader disclaimers.</v>
+        <v>Numerical fixes (LAYER_RATE, ILF_PARETO with xm, SWISSRE→Bernegger, AGGREGATE_TVAR); ExcelDna 1.9 + net8.0-windows; nullable seed; copula error handling.</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
-        <v>v0.3.1</v>
+        <v>v0.4.0</v>
       </c>
       <c r="B27" t="str">
-        <v>2026-02-21</v>
+        <v>2026-05-02</v>
       </c>
       <c r="C27" t="str">
-        <v>Aggregate Claims tab; spreadsheet rebuilt as .xlsx with full coverage.</v>
+        <v>GLM hat matrix bootstrap; Aggregate Claims formula fix; broader disclaimers.</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="str">
-        <v>v0.3.0</v>
+        <v>v0.3.1</v>
       </c>
       <c r="B28" t="str">
         <v>2026-02-21</v>
       </c>
       <c r="C28" t="str">
-        <v>Enhanced ODP Bootstrap (E&amp;V 2002); Cape Cod method; credibility removed.</v>
+        <v>Aggregate Claims tab; spreadsheet rebuilt as .xlsx with full coverage.</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="str">
-        <v>v0.2.0</v>
+        <v>v0.3.0</v>
       </c>
       <c r="B29" t="str">
-        <v>2026-02-04</v>
+        <v>2026-02-21</v>
       </c>
       <c r="C29" t="str">
-        <v>Panjer recursion; ZT/ZM distributions; Pareto III/IV; Inverse Gaussian; Loglogistic; cat modelling.</v>
+        <v>Enhanced ODP Bootstrap (E&amp;V 2002); Cape Cod method; credibility removed.</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="str">
+        <v>v0.2.0</v>
+      </c>
+      <c r="B30" t="str">
+        <v>2026-02-04</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Panjer recursion; ZT/ZM distributions; Pareto III/IV; Inverse Gaussian; Loglogistic; cat modelling.</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="str">
         <v>v0.1.0</v>
       </c>
-      <c r="B30" t="str">
+      <c r="B31" t="str">
         <v>2026-01-31</v>
       </c>
-      <c r="C30" t="str">
+      <c r="C31" t="str">
         <v>Initial tagged release: distributions, LEV, chain ladder, Mack, exposure curves.</v>
       </c>
     </row>
@@ -18607,7 +18618,7 @@
       </c>
       <c r="B304" t="str">
         <f>_xll.ACT_VERSION()</f>
-        <v>0.7.3</v>
+        <v>0.8.0</v>
       </c>
       <c r="C304" t="s">
         <v>350</v>
@@ -18619,7 +18630,7 @@
       </c>
       <c r="B305" t="str">
         <f>_xll.ACT_BUILD_DATE()</f>
-        <v>2026-05-04</v>
+        <v>2026-05-05</v>
       </c>
       <c r="C305" t="s">
         <v>352</v>
@@ -18643,7 +18654,7 @@
       </c>
       <c r="B307">
         <f>_xll.ACT_COMMIT_COUNT()</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C307" t="s">
         <v>356</v>
@@ -18655,7 +18666,7 @@
       </c>
       <c r="B308" t="str">
         <f>_xll.ACT_COMMIT_INFO(1, "hash")</f>
-        <v>v0.7.3</v>
+        <v>v0.8.0</v>
       </c>
       <c r="C308" t="s">
         <v>358</v>
@@ -18667,7 +18678,7 @@
       </c>
       <c r="B309" t="str">
         <f>_xll.ACT_COMMIT_INFO(1, "date")</f>
-        <v>2026-05-04</v>
+        <v>2026-05-05</v>
       </c>
       <c r="C309" t="s">
         <v>359</v>
@@ -18679,7 +18690,7 @@
       </c>
       <c r="B310" t="str">
         <f>_xll.ACT_COMMIT_INFO(1, "message")</f>
-        <v>Bundles five post-v0.7.2 fixes for the public surface: Cat Modeling SPILL collision (OEP/AEP curves now sit side-by-side with full 1000-row clearance, confused static Example 2 dropped); dump-iteration ordering (post-Formula2 errors now surface in dump JSON instead of silently shipping); Versions tab spills `=ACT_COMMIT_HISTORY()` live from the XLL instead of a stale `git log` snapshot; CHANGELOG.md / CONTRIBUTING.md / docs/DEVELOPING.md pulled out of the public repo (release notes live in this method + GitHub Releases).</v>
+        <v>Multi-target net48 + net8.0-windows. Default release asset (`AddIn64-packed.xll`) now targets .NET Framework 4.8 — preinstalled on every Windows 10 1903+ / Windows 11, so installing the add-in no longer requires a runtime download. A .NET 8 perf variant ships alongside as `AddIn64-packed-net8.xll` for users who install the .NET 8 Desktop Runtime; same C# code, modern JIT and SIMD codegen on heavy stochastic workloads. Root cause of the long-standing v0.5.x .NET 8 hosting failure identified: ExcelDna 1.9.0's host shim formats its own runtimeconfig.json from the `.dna` file's RuntimeVersion attribute, which was set to `v4.0` (causing the host to launch .NET 6 and reject the net8 user assembly). MSBuild XmlPoke target now rewrites it to `v8.0` for the net8 build only.</v>
       </c>
       <c r="C310" t="s">
         <v>360</v>
@@ -57588,11 +57599,11 @@
       </c>
       <c r="B312" s="3">
         <f>INDEX(_xll.ACT_COPULA_GUMBEL(B304, B305, B306), 4, 1)</f>
-        <v>0.35380375198453234</v>
+        <v>0.35380375198453229</v>
       </c>
       <c r="C312" s="3">
         <f>INDEX(_xll.ACT_COPULA_GUMBEL(B304, B305, B306), 4, 2)</f>
-        <v>0.2931304282767539</v>
+        <v>0.29313042827675378</v>
       </c>
     </row>
     <row r="313" spans="1:3" x14ac:dyDescent="0.25">
@@ -57839,7 +57850,7 @@
       </c>
       <c r="C331" s="3">
         <f>INDEX(_xll.ACT_COPULA_GUMBEL(B304, B305, B306), 23, 2)</f>
-        <v>0.60361747146042066</v>
+        <v>0.60361747146042077</v>
       </c>
     </row>
     <row r="332" spans="1:3" x14ac:dyDescent="0.25">
@@ -58030,11 +58041,11 @@
       </c>
       <c r="B346" s="3">
         <f>INDEX(_xll.ACT_COPULA_GUMBEL(B304, B305, B306), 38, 1)</f>
-        <v>0.14401509733294562</v>
+        <v>0.14401509733294554</v>
       </c>
       <c r="C346" s="3">
         <f>INDEX(_xll.ACT_COPULA_GUMBEL(B304, B305, B306), 38, 2)</f>
-        <v>6.1403171916247834E-2</v>
+        <v>6.1403171916247806E-2</v>
       </c>
     </row>
     <row r="347" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>